<commit_message>
Update README.md with new research paper reference for model implementation
</commit_message>
<xml_diff>
--- a/Checkpoints & Updates/Checkpoints.xlsx
+++ b/Checkpoints & Updates/Checkpoints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meghp\Desktop\Ahmedabad University\Term 1\CSE618 Artificial Intelligence Laboratory\Bird Species Detection\Checkpoints &amp; Updates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F9D002C-0C97-4664-829A-5F98157D63B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0895A187-73A5-4CC0-87C7-4864A8BE6797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Work Updates" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="305">
   <si>
     <t>Date</t>
   </si>
@@ -91,9 +91,6 @@
 4. Deleted folders for the species which are not considered</t>
   </si>
   <si>
-    <t>Get the range of the number of species for all the species considered/non-considered</t>
-  </si>
-  <si>
     <t>Species Number</t>
   </si>
   <si>
@@ -947,6 +944,19 @@
   </si>
   <si>
     <t>200</t>
+  </si>
+  <si>
+    <t>1. Data Segregation (Based on the updated list of species)</t>
+  </si>
+  <si>
+    <t>1. Updated bounded_boxes.txt manually as per the selected range of species [Converted to CSV and implemented the changes]</t>
+  </si>
+  <si>
+    <t>1. Updated train_test_split.txt manually as per the selected range of species [Converted to CSV and implemented the changes]</t>
+  </si>
+  <si>
+    <t>1. Get the range of the number of species for all the species considered/non-considered
+2. Implement Data Segregation in bounded_boxes.txt and train_test_split.txt</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1054,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1067,48 +1077,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1152,13 +1125,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1449,16 +1416,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="48.44140625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="86.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="55.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="106.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="105.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="71.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="64.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
@@ -1466,12 +1433,12 @@
       <c r="A1" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="17"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
@@ -1517,7 +1484,7 @@
       </c>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>45916</v>
       </c>
@@ -1533,12 +1500,33 @@
       <c r="E4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>45837</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="G5" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1563,19 +1551,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18.600000000000001" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18.600000000000001" x14ac:dyDescent="0.55000000000000004">
@@ -1583,7 +1571,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="11">
         <v>1</v>
@@ -1601,7 +1589,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C3" s="11">
         <f>D2+1</f>
@@ -1620,7 +1608,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="11">
         <f>D3+1</f>
@@ -1639,7 +1627,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="11">
         <f t="shared" ref="C5:C68" si="1">D4+1</f>
@@ -1658,7 +1646,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="11">
         <f t="shared" si="1"/>
@@ -1677,7 +1665,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="11">
         <f t="shared" si="1"/>
@@ -1696,7 +1684,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="11">
         <f t="shared" si="1"/>
@@ -1715,7 +1703,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" s="11">
         <f t="shared" si="1"/>
@@ -1734,7 +1722,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="11">
         <f t="shared" si="1"/>
@@ -1753,7 +1741,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C11" s="11">
         <f t="shared" si="1"/>
@@ -1772,7 +1760,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" s="11">
         <f t="shared" si="1"/>
@@ -1791,7 +1779,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="11">
         <f t="shared" si="1"/>
@@ -1810,7 +1798,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="11">
         <f t="shared" si="1"/>
@@ -1829,7 +1817,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C15" s="11">
         <f t="shared" si="1"/>
@@ -1848,7 +1836,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16" s="11">
         <f t="shared" si="1"/>
@@ -1867,7 +1855,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="11">
         <f t="shared" si="1"/>
@@ -1886,7 +1874,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="11">
         <f t="shared" si="1"/>
@@ -1905,7 +1893,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="11">
         <f t="shared" si="1"/>
@@ -1924,7 +1912,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="11">
         <f t="shared" si="1"/>
@@ -1943,7 +1931,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="11">
         <f t="shared" si="1"/>
@@ -1962,7 +1950,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="11">
         <f t="shared" si="1"/>
@@ -1981,7 +1969,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="11">
         <f t="shared" si="1"/>
@@ -2000,7 +1988,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24" s="11">
         <f t="shared" si="1"/>
@@ -2019,7 +2007,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" s="11">
         <f t="shared" si="1"/>
@@ -2038,7 +2026,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C26" s="11">
         <f t="shared" si="1"/>
@@ -2057,7 +2045,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C27" s="11">
         <f t="shared" si="1"/>
@@ -2076,7 +2064,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C28" s="11">
         <f t="shared" si="1"/>
@@ -2095,7 +2083,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" s="11">
         <f t="shared" si="1"/>
@@ -2114,7 +2102,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C30" s="11">
         <f t="shared" si="1"/>
@@ -2133,7 +2121,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C31" s="11">
         <f t="shared" si="1"/>
@@ -2152,7 +2140,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C32" s="11">
         <f t="shared" si="1"/>
@@ -2171,7 +2159,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C33" s="11">
         <f t="shared" si="1"/>
@@ -2190,7 +2178,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C34" s="11">
         <f t="shared" si="1"/>
@@ -2209,7 +2197,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C35" s="11">
         <f t="shared" si="1"/>
@@ -2228,7 +2216,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C36" s="11">
         <f t="shared" si="1"/>
@@ -2247,7 +2235,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C37" s="11">
         <f t="shared" si="1"/>
@@ -2266,7 +2254,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C38" s="11">
         <f t="shared" si="1"/>
@@ -2285,7 +2273,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C39" s="11">
         <f t="shared" si="1"/>
@@ -2304,10 +2292,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C40" s="11">
-        <f t="shared" si="1"/>
+        <f>D39+1</f>
         <v>2172</v>
       </c>
       <c r="D40" s="11">
@@ -2323,7 +2311,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C41" s="11">
         <f t="shared" si="1"/>
@@ -2342,7 +2330,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C42" s="11">
         <f t="shared" si="1"/>
@@ -2361,7 +2349,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C43" s="11">
         <f t="shared" si="1"/>
@@ -2380,7 +2368,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C44" s="11">
         <f t="shared" si="1"/>
@@ -2399,7 +2387,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C45" s="11">
         <f t="shared" si="1"/>
@@ -2418,7 +2406,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C46" s="11">
         <f t="shared" si="1"/>
@@ -2437,7 +2425,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C47" s="11">
         <f t="shared" si="1"/>
@@ -2456,7 +2444,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C48" s="11">
         <f t="shared" si="1"/>
@@ -2475,7 +2463,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C49" s="11">
         <f t="shared" si="1"/>
@@ -2494,7 +2482,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C50" s="11">
         <f t="shared" si="1"/>
@@ -2513,7 +2501,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C51" s="11">
         <f t="shared" si="1"/>
@@ -2532,7 +2520,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C52" s="11">
         <f t="shared" si="1"/>
@@ -2551,10 +2539,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C53" s="11">
-        <f t="shared" si="1"/>
+        <f>D52+1</f>
         <v>2950</v>
       </c>
       <c r="D53" s="11">
@@ -2570,7 +2558,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C54" s="11">
         <f t="shared" si="1"/>
@@ -2589,7 +2577,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C55" s="11">
         <f t="shared" si="1"/>
@@ -2608,7 +2596,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C56" s="11">
         <f t="shared" si="1"/>
@@ -2627,7 +2615,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C57" s="11">
         <f t="shared" si="1"/>
@@ -2646,7 +2634,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C58" s="11">
         <f t="shared" si="1"/>
@@ -2665,7 +2653,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C59" s="11">
         <f t="shared" si="1"/>
@@ -2684,10 +2672,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C60" s="11">
-        <f t="shared" si="1"/>
+        <f>D59+1</f>
         <v>3368</v>
       </c>
       <c r="D60" s="11">
@@ -2703,7 +2691,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C61" s="11">
         <f t="shared" si="1"/>
@@ -2722,7 +2710,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C62" s="11">
         <f t="shared" si="1"/>
@@ -2741,7 +2729,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C63" s="11">
         <f t="shared" si="1"/>
@@ -2760,7 +2748,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="11" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C64" s="11">
         <f t="shared" si="1"/>
@@ -2779,7 +2767,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="11" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C65" s="11">
         <f t="shared" si="1"/>
@@ -2798,7 +2786,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="11" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C66" s="11">
         <f t="shared" si="1"/>
@@ -2817,7 +2805,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C67" s="11">
         <f t="shared" si="1"/>
@@ -2836,7 +2824,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C68" s="11">
         <f t="shared" si="1"/>
@@ -2855,7 +2843,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C69" s="11">
         <f t="shared" ref="C69:C132" si="3">D68+1</f>
@@ -2874,7 +2862,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C70" s="11">
         <f t="shared" si="3"/>
@@ -2893,7 +2881,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C71" s="11">
         <f t="shared" si="3"/>
@@ -2912,7 +2900,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C72" s="11">
         <f t="shared" si="3"/>
@@ -2931,7 +2919,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C73" s="11">
         <f t="shared" si="3"/>
@@ -2950,7 +2938,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C74" s="11">
         <f t="shared" si="3"/>
@@ -2969,7 +2957,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C75" s="11">
         <f t="shared" si="3"/>
@@ -2988,7 +2976,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C76" s="11">
         <f t="shared" si="3"/>
@@ -3007,7 +2995,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C77" s="11">
         <f t="shared" si="3"/>
@@ -3026,7 +3014,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C78" s="11">
         <f t="shared" si="3"/>
@@ -3045,7 +3033,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C79" s="11">
         <f t="shared" si="3"/>
@@ -3064,7 +3052,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C80" s="11">
         <f t="shared" si="3"/>
@@ -3083,7 +3071,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C81" s="11">
         <f t="shared" si="3"/>
@@ -3102,7 +3090,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C82" s="11">
         <f t="shared" si="3"/>
@@ -3121,7 +3109,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C83" s="11">
         <f t="shared" si="3"/>
@@ -3140,7 +3128,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C84" s="11">
         <f t="shared" si="3"/>
@@ -3159,7 +3147,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C85" s="11">
         <f t="shared" si="3"/>
@@ -3178,7 +3166,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C86" s="11">
         <f t="shared" si="3"/>
@@ -3197,7 +3185,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C87" s="11">
         <f t="shared" si="3"/>
@@ -3216,7 +3204,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C88" s="11">
         <f t="shared" si="3"/>
@@ -3235,7 +3223,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C89" s="11">
         <f t="shared" si="3"/>
@@ -3254,7 +3242,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C90" s="11">
         <f t="shared" si="3"/>
@@ -3273,7 +3261,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C91" s="11">
         <f t="shared" si="3"/>
@@ -3292,7 +3280,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C92" s="11">
         <f t="shared" si="3"/>
@@ -3311,7 +3299,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C93" s="11">
         <f t="shared" si="3"/>
@@ -3330,7 +3318,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C94" s="11">
         <f t="shared" si="3"/>
@@ -3349,7 +3337,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C95" s="11">
         <f t="shared" si="3"/>
@@ -3368,7 +3356,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C96" s="11">
         <f t="shared" si="3"/>
@@ -3387,7 +3375,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="11" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C97" s="11">
         <f t="shared" si="3"/>
@@ -3406,7 +3394,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C98" s="11">
         <f t="shared" si="3"/>
@@ -3425,7 +3413,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C99" s="11">
         <f t="shared" si="3"/>
@@ -3444,7 +3432,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C100" s="11">
         <f t="shared" si="3"/>
@@ -3463,7 +3451,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C101" s="11">
         <f t="shared" si="3"/>
@@ -3482,7 +3470,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C102" s="11">
         <f t="shared" si="3"/>
@@ -3501,7 +3489,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C103" s="11">
         <f t="shared" si="3"/>
@@ -3520,7 +3508,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C104" s="11">
         <f t="shared" si="3"/>
@@ -3539,7 +3527,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C105" s="11">
         <f t="shared" si="3"/>
@@ -3558,7 +3546,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C106" s="11">
         <f t="shared" si="3"/>
@@ -3577,7 +3565,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C107" s="11">
         <f t="shared" si="3"/>
@@ -3596,7 +3584,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C108" s="11">
         <f t="shared" si="3"/>
@@ -3615,7 +3603,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C109" s="11">
         <f t="shared" si="3"/>
@@ -3634,7 +3622,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C110" s="11">
         <f t="shared" si="3"/>
@@ -3653,7 +3641,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C111" s="11">
         <f t="shared" si="3"/>
@@ -3672,7 +3660,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C112" s="11">
         <f t="shared" si="3"/>
@@ -3691,7 +3679,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C113" s="11">
         <f t="shared" si="3"/>
@@ -3710,10 +3698,10 @@
         <v>113</v>
       </c>
       <c r="B114" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C114" s="11">
-        <f t="shared" si="3"/>
+        <f>D113+1</f>
         <v>6563</v>
       </c>
       <c r="D114" s="11">
@@ -3729,7 +3717,7 @@
         <v>114</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C115" s="11">
         <f t="shared" si="3"/>
@@ -3748,7 +3736,7 @@
         <v>115</v>
       </c>
       <c r="B116" s="11" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C116" s="11">
         <f t="shared" si="3"/>
@@ -3767,7 +3755,7 @@
         <v>116</v>
       </c>
       <c r="B117" s="11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C117" s="11">
         <f t="shared" si="3"/>
@@ -3786,7 +3774,7 @@
         <v>117</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C118" s="11">
         <f t="shared" si="3"/>
@@ -3805,7 +3793,7 @@
         <v>118</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C119" s="11">
         <f t="shared" si="3"/>
@@ -3824,7 +3812,7 @@
         <v>119</v>
       </c>
       <c r="B120" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C120" s="11">
         <f t="shared" si="3"/>
@@ -3843,7 +3831,7 @@
         <v>120</v>
       </c>
       <c r="B121" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C121" s="11">
         <f t="shared" si="3"/>
@@ -3862,7 +3850,7 @@
         <v>121</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C122" s="11">
         <f t="shared" si="3"/>
@@ -3881,7 +3869,7 @@
         <v>122</v>
       </c>
       <c r="B123" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C123" s="11">
         <f t="shared" si="3"/>
@@ -3900,7 +3888,7 @@
         <v>123</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C124" s="11">
         <f t="shared" si="3"/>
@@ -3919,7 +3907,7 @@
         <v>124</v>
       </c>
       <c r="B125" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C125" s="11">
         <f t="shared" si="3"/>
@@ -3938,7 +3926,7 @@
         <v>125</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C126" s="11">
         <f t="shared" si="3"/>
@@ -3957,7 +3945,7 @@
         <v>126</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C127" s="11">
         <f t="shared" si="3"/>
@@ -3976,7 +3964,7 @@
         <v>127</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C128" s="11">
         <f t="shared" si="3"/>
@@ -3995,7 +3983,7 @@
         <v>128</v>
       </c>
       <c r="B129" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C129" s="11">
         <f t="shared" si="3"/>
@@ -4014,7 +4002,7 @@
         <v>129</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C130" s="11">
         <f t="shared" si="3"/>
@@ -4033,7 +4021,7 @@
         <v>130</v>
       </c>
       <c r="B131" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C131" s="11">
         <f t="shared" si="3"/>
@@ -4052,7 +4040,7 @@
         <v>131</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C132" s="11">
         <f t="shared" si="3"/>
@@ -4071,7 +4059,7 @@
         <v>132</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C133" s="11">
         <f t="shared" ref="C133:C196" si="5">D132+1</f>
@@ -4090,7 +4078,7 @@
         <v>133</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C134" s="11">
         <f t="shared" si="5"/>
@@ -4109,7 +4097,7 @@
         <v>134</v>
       </c>
       <c r="B135" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C135" s="11">
         <f t="shared" si="5"/>
@@ -4128,7 +4116,7 @@
         <v>135</v>
       </c>
       <c r="B136" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C136" s="11">
         <f t="shared" si="5"/>
@@ -4147,7 +4135,7 @@
         <v>136</v>
       </c>
       <c r="B137" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C137" s="11">
         <f t="shared" si="5"/>
@@ -4166,7 +4154,7 @@
         <v>137</v>
       </c>
       <c r="B138" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C138" s="11">
         <f t="shared" si="5"/>
@@ -4185,7 +4173,7 @@
         <v>138</v>
       </c>
       <c r="B139" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C139" s="11">
         <f t="shared" si="5"/>
@@ -4204,7 +4192,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C140" s="11">
         <f t="shared" si="5"/>
@@ -4223,7 +4211,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C141" s="11">
         <f t="shared" si="5"/>
@@ -4242,7 +4230,7 @@
         <v>141</v>
       </c>
       <c r="B142" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C142" s="11">
         <f t="shared" si="5"/>
@@ -4261,7 +4249,7 @@
         <v>142</v>
       </c>
       <c r="B143" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C143" s="11">
         <f t="shared" si="5"/>
@@ -4280,7 +4268,7 @@
         <v>143</v>
       </c>
       <c r="B144" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C144" s="11">
         <f t="shared" si="5"/>
@@ -4299,7 +4287,7 @@
         <v>144</v>
       </c>
       <c r="B145" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C145" s="11">
         <f t="shared" si="5"/>
@@ -4318,7 +4306,7 @@
         <v>145</v>
       </c>
       <c r="B146" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C146" s="11">
         <f t="shared" si="5"/>
@@ -4337,7 +4325,7 @@
         <v>146</v>
       </c>
       <c r="B147" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C147" s="11">
         <f t="shared" si="5"/>
@@ -4356,7 +4344,7 @@
         <v>147</v>
       </c>
       <c r="B148" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C148" s="11">
         <f t="shared" si="5"/>
@@ -4375,7 +4363,7 @@
         <v>148</v>
       </c>
       <c r="B149" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C149" s="11">
         <f t="shared" si="5"/>
@@ -4394,7 +4382,7 @@
         <v>149</v>
       </c>
       <c r="B150" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C150" s="11">
         <f t="shared" si="5"/>
@@ -4413,7 +4401,7 @@
         <v>150</v>
       </c>
       <c r="B151" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C151" s="11">
         <f t="shared" si="5"/>
@@ -4432,7 +4420,7 @@
         <v>151</v>
       </c>
       <c r="B152" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C152" s="11">
         <f t="shared" si="5"/>
@@ -4451,10 +4439,10 @@
         <v>152</v>
       </c>
       <c r="B153" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C153" s="11">
-        <f t="shared" si="5"/>
+        <f>D152+1</f>
         <v>8874</v>
       </c>
       <c r="D153" s="11">
@@ -4470,7 +4458,7 @@
         <v>153</v>
       </c>
       <c r="B154" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C154" s="11">
         <f t="shared" si="5"/>
@@ -4489,7 +4477,7 @@
         <v>154</v>
       </c>
       <c r="B155" s="11" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C155" s="11">
         <f t="shared" si="5"/>
@@ -4508,7 +4496,7 @@
         <v>155</v>
       </c>
       <c r="B156" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C156" s="11">
         <f t="shared" si="5"/>
@@ -4527,7 +4515,7 @@
         <v>156</v>
       </c>
       <c r="B157" s="11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C157" s="11">
         <f t="shared" si="5"/>
@@ -4546,7 +4534,7 @@
         <v>157</v>
       </c>
       <c r="B158" s="11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C158" s="11">
         <f t="shared" si="5"/>
@@ -4565,7 +4553,7 @@
         <v>158</v>
       </c>
       <c r="B159" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C159" s="11">
         <f t="shared" si="5"/>
@@ -4584,7 +4572,7 @@
         <v>159</v>
       </c>
       <c r="B160" s="11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C160" s="11">
         <f t="shared" si="5"/>
@@ -4603,7 +4591,7 @@
         <v>160</v>
       </c>
       <c r="B161" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C161" s="11">
         <f t="shared" si="5"/>
@@ -4622,7 +4610,7 @@
         <v>161</v>
       </c>
       <c r="B162" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C162" s="11">
         <f t="shared" si="5"/>
@@ -4641,7 +4629,7 @@
         <v>162</v>
       </c>
       <c r="B163" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C163" s="11">
         <f t="shared" si="5"/>
@@ -4660,7 +4648,7 @@
         <v>163</v>
       </c>
       <c r="B164" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C164" s="11">
         <f t="shared" si="5"/>
@@ -4679,7 +4667,7 @@
         <v>164</v>
       </c>
       <c r="B165" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C165" s="11">
         <f t="shared" si="5"/>
@@ -4698,7 +4686,7 @@
         <v>165</v>
       </c>
       <c r="B166" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C166" s="11">
         <f t="shared" si="5"/>
@@ -4717,7 +4705,7 @@
         <v>166</v>
       </c>
       <c r="B167" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C167" s="11">
         <f t="shared" si="5"/>
@@ -4736,7 +4724,7 @@
         <v>167</v>
       </c>
       <c r="B168" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C168" s="11">
         <f t="shared" si="5"/>
@@ -4755,7 +4743,7 @@
         <v>168</v>
       </c>
       <c r="B169" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C169" s="11">
         <f t="shared" si="5"/>
@@ -4774,7 +4762,7 @@
         <v>169</v>
       </c>
       <c r="B170" s="11" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C170" s="11">
         <f t="shared" si="5"/>
@@ -4793,7 +4781,7 @@
         <v>170</v>
       </c>
       <c r="B171" s="11" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C171" s="11">
         <f t="shared" si="5"/>
@@ -4812,7 +4800,7 @@
         <v>171</v>
       </c>
       <c r="B172" s="11" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C172" s="11">
         <f t="shared" si="5"/>
@@ -4831,7 +4819,7 @@
         <v>172</v>
       </c>
       <c r="B173" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C173" s="11">
         <f t="shared" si="5"/>
@@ -4850,7 +4838,7 @@
         <v>173</v>
       </c>
       <c r="B174" s="11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C174" s="11">
         <f t="shared" si="5"/>
@@ -4869,7 +4857,7 @@
         <v>174</v>
       </c>
       <c r="B175" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C175" s="11">
         <f t="shared" si="5"/>
@@ -4888,7 +4876,7 @@
         <v>175</v>
       </c>
       <c r="B176" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C176" s="11">
         <f t="shared" si="5"/>
@@ -4907,7 +4895,7 @@
         <v>176</v>
       </c>
       <c r="B177" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C177" s="11">
         <f t="shared" si="5"/>
@@ -4926,7 +4914,7 @@
         <v>177</v>
       </c>
       <c r="B178" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C178" s="11">
         <f t="shared" si="5"/>
@@ -4945,7 +4933,7 @@
         <v>178</v>
       </c>
       <c r="B179" s="11" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C179" s="11">
         <f t="shared" si="5"/>
@@ -4964,7 +4952,7 @@
         <v>179</v>
       </c>
       <c r="B180" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C180" s="11">
         <f t="shared" si="5"/>
@@ -4983,7 +4971,7 @@
         <v>180</v>
       </c>
       <c r="B181" s="11" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C181" s="11">
         <f t="shared" si="5"/>
@@ -5002,7 +4990,7 @@
         <v>181</v>
       </c>
       <c r="B182" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C182" s="11">
         <f t="shared" si="5"/>
@@ -5021,7 +5009,7 @@
         <v>182</v>
       </c>
       <c r="B183" s="11" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C183" s="11">
         <f t="shared" si="5"/>
@@ -5040,7 +5028,7 @@
         <v>183</v>
       </c>
       <c r="B184" s="11" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C184" s="11">
         <f t="shared" si="5"/>
@@ -5059,7 +5047,7 @@
         <v>184</v>
       </c>
       <c r="B185" s="11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C185" s="11">
         <f t="shared" si="5"/>
@@ -5078,7 +5066,7 @@
         <v>185</v>
       </c>
       <c r="B186" s="11" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C186" s="11">
         <f t="shared" si="5"/>
@@ -5097,7 +5085,7 @@
         <v>186</v>
       </c>
       <c r="B187" s="11" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C187" s="11">
         <f t="shared" si="5"/>
@@ -5116,7 +5104,7 @@
         <v>187</v>
       </c>
       <c r="B188" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C188" s="11">
         <f t="shared" si="5"/>
@@ -5135,7 +5123,7 @@
         <v>188</v>
       </c>
       <c r="B189" s="11" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C189" s="11">
         <f t="shared" si="5"/>
@@ -5154,7 +5142,7 @@
         <v>189</v>
       </c>
       <c r="B190" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C190" s="11">
         <f t="shared" si="5"/>
@@ -5173,7 +5161,7 @@
         <v>190</v>
       </c>
       <c r="B191" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C191" s="11">
         <f t="shared" si="5"/>
@@ -5192,7 +5180,7 @@
         <v>191</v>
       </c>
       <c r="B192" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C192" s="11">
         <f t="shared" si="5"/>
@@ -5211,7 +5199,7 @@
         <v>192</v>
       </c>
       <c r="B193" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C193" s="11">
         <f t="shared" si="5"/>
@@ -5230,7 +5218,7 @@
         <v>193</v>
       </c>
       <c r="B194" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C194" s="11">
         <f t="shared" si="5"/>
@@ -5249,7 +5237,7 @@
         <v>194</v>
       </c>
       <c r="B195" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C195" s="11">
         <f t="shared" si="5"/>
@@ -5268,7 +5256,7 @@
         <v>195</v>
       </c>
       <c r="B196" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C196" s="11">
         <f t="shared" si="5"/>
@@ -5287,7 +5275,7 @@
         <v>196</v>
       </c>
       <c r="B197" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C197" s="11">
         <f t="shared" ref="C197:C201" si="7">D196+1</f>
@@ -5306,7 +5294,7 @@
         <v>197</v>
       </c>
       <c r="B198" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C198" s="11">
         <f t="shared" si="7"/>
@@ -5325,7 +5313,7 @@
         <v>198</v>
       </c>
       <c r="B199" s="11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C199" s="11">
         <f t="shared" si="7"/>
@@ -5344,7 +5332,7 @@
         <v>199</v>
       </c>
       <c r="B200" s="11" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C200" s="11">
         <f t="shared" si="7"/>
@@ -5363,7 +5351,7 @@
         <v>200</v>
       </c>
       <c r="B201" s="11" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C201" s="11">
         <f t="shared" si="7"/>
@@ -5424,402 +5412,402 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="14" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="14" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="14" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="14" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" s="14" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" s="14" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="14" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="14" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="14" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="14" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="14" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="14" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" s="14" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" s="14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" s="14" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" s="14" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="14" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" s="14" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" s="14" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" s="14" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="14" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" s="14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" s="14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" s="14" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" s="14" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" s="14" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" s="14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" s="14" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="14" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="14" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" s="14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" s="14" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="14" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" s="14" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" s="14" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" s="14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" s="14" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A62" s="14" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A63" s="14" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A64" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A65" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A66" s="14" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A67" s="14" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A68" s="14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A69" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A70" s="14" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A71" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A72" s="14" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A73" s="14" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A74" s="14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A75" s="14" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A76" s="14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A77" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A78" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A79" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A80" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>